<commit_message>
publish: 2026-09-08 14:21 BST
</commit_message>
<xml_diff>
--- a/files/Downloads/Week 7/Regression_Calculations_Week 7.xlsx
+++ b/files/Downloads/Week 7/Regression_Calculations_Week 7.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u1373867/Dropbox/PO12Q/files/Downloads/Week 7/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2D12E2-2FB4-C44B-AF30-F1F7788A8227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533D64DA-2904-5649-80D5-08E06BB453DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="660" windowWidth="27820" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1083,14 +1083,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -1236,10 +1233,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" b="0" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -1388,14 +1382,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -1725,14 +1716,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -1914,10 +1902,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" b="0" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -2114,15 +2099,12 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:acc>
                       <m:accPr>
                         <m:chr m:val="̂"/>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2254,15 +2236,12 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:acc>
                       <m:accPr>
                         <m:chr m:val="̂"/>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2418,14 +2397,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2441,7 +2417,7 @@
                           <m:accPr>
                             <m:chr m:val="̂"/>
                             <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1100" i="1">
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
                             </m:ctrlPr>
@@ -2619,10 +2595,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" b="0" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -2639,7 +2612,7 @@
                       <m:accPr>
                         <m:chr m:val="̂"/>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2777,14 +2750,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -2812,7 +2782,7 @@
                           <m:accPr>
                             <m:chr m:val="̂"/>
                             <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1100" i="1">
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
                             </m:ctrlPr>
@@ -2966,14 +2936,11 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
                         </m:ctrlPr>
@@ -3487,47 +3454,47 @@
         <v>650</v>
       </c>
       <c r="D3" s="4">
-        <f t="shared" ref="D3:D11" si="0">C3-$C$13</f>
+        <f>C3-$C$13</f>
         <v>-845</v>
       </c>
       <c r="E3" s="4">
-        <f t="shared" ref="E3:E11" si="1">D3^2</f>
+        <f t="shared" ref="E3:E11" si="0">D3^2</f>
         <v>714025</v>
       </c>
       <c r="F3" s="4">
-        <f t="shared" ref="F3:F11" si="2">B3-$B$13</f>
+        <f>B3-$B$13</f>
         <v>-20</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G11" si="3">F3^2</f>
+        <f t="shared" ref="G3:G11" si="1">F3^2</f>
         <v>400</v>
       </c>
       <c r="H3" s="4">
-        <f t="shared" ref="H3:H11" si="4">D3*F3</f>
+        <f t="shared" ref="H3:H11" si="2">D3*F3</f>
         <v>16900</v>
       </c>
       <c r="I3" s="4">
-        <f t="shared" ref="I3:I11" si="5">-53.1+39.7*B3</f>
+        <f t="shared" ref="I3:I11" si="3">-53.1+39.7*B3</f>
         <v>701.2</v>
       </c>
       <c r="J3" s="4">
-        <f t="shared" ref="J3:J11" si="6">I3-$C$13</f>
+        <f>I3-$C$13</f>
         <v>-793.8</v>
       </c>
       <c r="K3" s="4">
-        <f t="shared" ref="K3:K11" si="7">J3^2</f>
+        <f t="shared" ref="K3:K11" si="4">J3^2</f>
         <v>630118.43999999994</v>
       </c>
       <c r="L3" s="4">
-        <f t="shared" ref="L3:L11" si="8">C3-I3</f>
+        <f t="shared" ref="L3:L11" si="5">C3-I3</f>
         <v>-51.200000000000045</v>
       </c>
       <c r="M3" s="4">
-        <f t="shared" ref="M3:M11" si="9">L3^2</f>
+        <f t="shared" ref="M3:M11" si="6">L3^2</f>
         <v>2621.4400000000046</v>
       </c>
       <c r="N3" s="4">
-        <f t="shared" ref="N3:N11" si="10">B3^2</f>
+        <f t="shared" ref="N3:N11" si="7">B3^2</f>
         <v>361</v>
       </c>
     </row>
@@ -3542,47 +3509,47 @@
         <v>2300</v>
       </c>
       <c r="D4" s="4">
+        <f>C4-$C$13</f>
+        <v>805</v>
+      </c>
+      <c r="E4" s="4">
         <f t="shared" si="0"/>
-        <v>805</v>
-      </c>
-      <c r="E4" s="4">
+        <v>648025</v>
+      </c>
+      <c r="F4" s="4">
+        <f>B4-$B$13</f>
+        <v>17</v>
+      </c>
+      <c r="G4" s="4">
         <f t="shared" si="1"/>
-        <v>648025</v>
-      </c>
-      <c r="F4" s="4">
+        <v>289</v>
+      </c>
+      <c r="H4" s="4">
         <f t="shared" si="2"/>
-        <v>17</v>
-      </c>
-      <c r="G4" s="4">
+        <v>13685</v>
+      </c>
+      <c r="I4" s="4">
         <f t="shared" si="3"/>
-        <v>289</v>
-      </c>
-      <c r="H4" s="4">
+        <v>2170.1000000000004</v>
+      </c>
+      <c r="J4" s="4">
+        <f>I4-$C$13</f>
+        <v>675.10000000000036</v>
+      </c>
+      <c r="K4" s="4">
         <f t="shared" si="4"/>
-        <v>13685</v>
-      </c>
-      <c r="I4" s="4">
+        <v>455760.01000000047</v>
+      </c>
+      <c r="L4" s="4">
         <f t="shared" si="5"/>
-        <v>2170.1000000000004</v>
-      </c>
-      <c r="J4" s="4">
+        <v>129.89999999999964</v>
+      </c>
+      <c r="M4" s="4">
         <f t="shared" si="6"/>
-        <v>675.10000000000036</v>
-      </c>
-      <c r="K4" s="4">
+        <v>16874.009999999904</v>
+      </c>
+      <c r="N4" s="4">
         <f t="shared" si="7"/>
-        <v>455760.01000000047</v>
-      </c>
-      <c r="L4" s="4">
-        <f t="shared" si="8"/>
-        <v>129.89999999999964</v>
-      </c>
-      <c r="M4" s="4">
-        <f t="shared" si="9"/>
-        <v>16874.009999999904</v>
-      </c>
-      <c r="N4" s="4">
-        <f t="shared" si="10"/>
         <v>3136</v>
       </c>
     </row>
@@ -3597,47 +3564,47 @@
         <v>1900</v>
       </c>
       <c r="D5" s="4">
+        <f>C5-$C$13</f>
+        <v>405</v>
+      </c>
+      <c r="E5" s="4">
         <f t="shared" si="0"/>
-        <v>405</v>
-      </c>
-      <c r="E5" s="4">
+        <v>164025</v>
+      </c>
+      <c r="F5" s="4">
+        <f>B5-$B$13</f>
+        <v>6</v>
+      </c>
+      <c r="G5" s="4">
         <f t="shared" si="1"/>
-        <v>164025</v>
-      </c>
-      <c r="F5" s="4">
+        <v>36</v>
+      </c>
+      <c r="H5" s="4">
         <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="G5" s="4">
+        <v>2430</v>
+      </c>
+      <c r="I5" s="4">
         <f t="shared" si="3"/>
-        <v>36</v>
-      </c>
-      <c r="H5" s="4">
+        <v>1733.4000000000003</v>
+      </c>
+      <c r="J5" s="4">
+        <f>I5-$C$13</f>
+        <v>238.40000000000032</v>
+      </c>
+      <c r="K5" s="4">
         <f t="shared" si="4"/>
-        <v>2430</v>
-      </c>
-      <c r="I5" s="4">
+        <v>56834.56000000015</v>
+      </c>
+      <c r="L5" s="4">
         <f t="shared" si="5"/>
-        <v>1733.4000000000003</v>
-      </c>
-      <c r="J5" s="4">
+        <v>166.59999999999968</v>
+      </c>
+      <c r="M5" s="4">
         <f t="shared" si="6"/>
-        <v>238.40000000000032</v>
-      </c>
-      <c r="K5" s="4">
+        <v>27755.559999999892</v>
+      </c>
+      <c r="N5" s="4">
         <f t="shared" si="7"/>
-        <v>56834.56000000015</v>
-      </c>
-      <c r="L5" s="4">
-        <f t="shared" si="8"/>
-        <v>166.59999999999968</v>
-      </c>
-      <c r="M5" s="4">
-        <f t="shared" si="9"/>
-        <v>27755.559999999892</v>
-      </c>
-      <c r="N5" s="4">
-        <f t="shared" si="10"/>
         <v>2025</v>
       </c>
     </row>
@@ -3652,47 +3619,47 @@
         <v>2000</v>
       </c>
       <c r="D6" s="4">
+        <f>C6-$C$13</f>
+        <v>505</v>
+      </c>
+      <c r="E6" s="4">
         <f t="shared" si="0"/>
-        <v>505</v>
-      </c>
-      <c r="E6" s="4">
+        <v>255025</v>
+      </c>
+      <c r="F6" s="4">
+        <f>B6-$B$13</f>
+        <v>-2</v>
+      </c>
+      <c r="G6" s="4">
         <f t="shared" si="1"/>
-        <v>255025</v>
-      </c>
-      <c r="F6" s="4">
+        <v>4</v>
+      </c>
+      <c r="H6" s="4">
         <f t="shared" si="2"/>
-        <v>-2</v>
-      </c>
-      <c r="G6" s="4">
+        <v>-1010</v>
+      </c>
+      <c r="I6" s="4">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="H6" s="4">
+        <v>1415.8000000000002</v>
+      </c>
+      <c r="J6" s="4">
+        <f>I6-$C$13</f>
+        <v>-79.199999999999818</v>
+      </c>
+      <c r="K6" s="4">
         <f t="shared" si="4"/>
-        <v>-1010</v>
-      </c>
-      <c r="I6" s="4">
+        <v>6272.6399999999712</v>
+      </c>
+      <c r="L6" s="4">
         <f t="shared" si="5"/>
-        <v>1415.8000000000002</v>
-      </c>
-      <c r="J6" s="4">
+        <v>584.19999999999982</v>
+      </c>
+      <c r="M6" s="4">
         <f t="shared" si="6"/>
-        <v>-79.199999999999818</v>
-      </c>
-      <c r="K6" s="4">
+        <v>341289.63999999978</v>
+      </c>
+      <c r="N6" s="4">
         <f t="shared" si="7"/>
-        <v>6272.6399999999712</v>
-      </c>
-      <c r="L6" s="4">
-        <f t="shared" si="8"/>
-        <v>584.19999999999982</v>
-      </c>
-      <c r="M6" s="4">
-        <f t="shared" si="9"/>
-        <v>341289.63999999978</v>
-      </c>
-      <c r="N6" s="4">
-        <f t="shared" si="10"/>
         <v>1369</v>
       </c>
     </row>
@@ -3707,47 +3674,47 @@
         <v>900</v>
       </c>
       <c r="D7" s="4">
+        <f t="shared" ref="D7:D11" si="8">C7-$C$13</f>
+        <v>-595</v>
+      </c>
+      <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v>-595</v>
-      </c>
-      <c r="E7" s="4">
+        <v>354025</v>
+      </c>
+      <c r="F7" s="4">
+        <f t="shared" ref="F7:F11" si="9">B7-$B$13</f>
+        <v>-16</v>
+      </c>
+      <c r="G7" s="4">
         <f t="shared" si="1"/>
-        <v>354025</v>
-      </c>
-      <c r="F7" s="4">
+        <v>256</v>
+      </c>
+      <c r="H7" s="4">
         <f t="shared" si="2"/>
-        <v>-16</v>
-      </c>
-      <c r="G7" s="4">
+        <v>9520</v>
+      </c>
+      <c r="I7" s="4">
         <f t="shared" si="3"/>
-        <v>256</v>
-      </c>
-      <c r="H7" s="4">
+        <v>860</v>
+      </c>
+      <c r="J7" s="4">
+        <f t="shared" ref="J7:J11" si="10">I7-$C$13</f>
+        <v>-635</v>
+      </c>
+      <c r="K7" s="4">
         <f t="shared" si="4"/>
-        <v>9520</v>
-      </c>
-      <c r="I7" s="4">
+        <v>403225</v>
+      </c>
+      <c r="L7" s="4">
         <f t="shared" si="5"/>
-        <v>860</v>
-      </c>
-      <c r="J7" s="4">
+        <v>40</v>
+      </c>
+      <c r="M7" s="4">
         <f t="shared" si="6"/>
-        <v>-635</v>
-      </c>
-      <c r="K7" s="4">
+        <v>1600</v>
+      </c>
+      <c r="N7" s="4">
         <f t="shared" si="7"/>
-        <v>403225</v>
-      </c>
-      <c r="L7" s="4">
-        <f t="shared" si="8"/>
-        <v>40</v>
-      </c>
-      <c r="M7" s="4">
-        <f t="shared" si="9"/>
-        <v>1600</v>
-      </c>
-      <c r="N7" s="4">
-        <f t="shared" si="10"/>
         <v>529</v>
       </c>
     </row>
@@ -3762,47 +3729,47 @@
         <v>1000</v>
       </c>
       <c r="D8" s="4">
+        <f t="shared" si="8"/>
+        <v>-495</v>
+      </c>
+      <c r="E8" s="4">
         <f t="shared" si="0"/>
-        <v>-495</v>
-      </c>
-      <c r="E8" s="4">
+        <v>245025</v>
+      </c>
+      <c r="F8" s="4">
+        <f t="shared" si="9"/>
+        <v>-7</v>
+      </c>
+      <c r="G8" s="4">
         <f t="shared" si="1"/>
-        <v>245025</v>
-      </c>
-      <c r="F8" s="4">
+        <v>49</v>
+      </c>
+      <c r="H8" s="4">
         <f t="shared" si="2"/>
-        <v>-7</v>
-      </c>
-      <c r="G8" s="4">
+        <v>3465</v>
+      </c>
+      <c r="I8" s="4">
         <f t="shared" si="3"/>
-        <v>49</v>
-      </c>
-      <c r="H8" s="4">
+        <v>1217.3000000000002</v>
+      </c>
+      <c r="J8" s="4">
+        <f t="shared" si="10"/>
+        <v>-277.69999999999982</v>
+      </c>
+      <c r="K8" s="4">
         <f t="shared" si="4"/>
-        <v>3465</v>
-      </c>
-      <c r="I8" s="4">
+        <v>77117.289999999892</v>
+      </c>
+      <c r="L8" s="4">
         <f t="shared" si="5"/>
-        <v>1217.3000000000002</v>
-      </c>
-      <c r="J8" s="4">
+        <v>-217.30000000000018</v>
+      </c>
+      <c r="M8" s="4">
         <f t="shared" si="6"/>
-        <v>-277.69999999999982</v>
-      </c>
-      <c r="K8" s="4">
+        <v>47219.290000000081</v>
+      </c>
+      <c r="N8" s="4">
         <f t="shared" si="7"/>
-        <v>77117.289999999892</v>
-      </c>
-      <c r="L8" s="4">
-        <f t="shared" si="8"/>
-        <v>-217.30000000000018</v>
-      </c>
-      <c r="M8" s="4">
-        <f t="shared" si="9"/>
-        <v>47219.290000000081</v>
-      </c>
-      <c r="N8" s="4">
-        <f t="shared" si="10"/>
         <v>1024</v>
       </c>
     </row>
@@ -3817,47 +3784,47 @@
         <v>2500</v>
       </c>
       <c r="D9" s="4">
+        <f t="shared" si="8"/>
+        <v>1005</v>
+      </c>
+      <c r="E9" s="4">
         <f t="shared" si="0"/>
-        <v>1005</v>
-      </c>
-      <c r="E9" s="4">
+        <v>1010025</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="9"/>
+        <v>26</v>
+      </c>
+      <c r="G9" s="4">
         <f t="shared" si="1"/>
-        <v>1010025</v>
-      </c>
-      <c r="F9" s="4">
+        <v>676</v>
+      </c>
+      <c r="H9" s="4">
         <f t="shared" si="2"/>
-        <v>26</v>
-      </c>
-      <c r="G9" s="4">
+        <v>26130</v>
+      </c>
+      <c r="I9" s="4">
         <f t="shared" si="3"/>
-        <v>676</v>
-      </c>
-      <c r="H9" s="4">
+        <v>2527.4</v>
+      </c>
+      <c r="J9" s="4">
+        <f t="shared" si="10"/>
+        <v>1032.4000000000001</v>
+      </c>
+      <c r="K9" s="4">
         <f t="shared" si="4"/>
-        <v>26130</v>
-      </c>
-      <c r="I9" s="4">
+        <v>1065849.7600000002</v>
+      </c>
+      <c r="L9" s="4">
         <f t="shared" si="5"/>
-        <v>2527.4</v>
-      </c>
-      <c r="J9" s="4">
+        <v>-27.400000000000091</v>
+      </c>
+      <c r="M9" s="4">
         <f t="shared" si="6"/>
-        <v>1032.4000000000001</v>
-      </c>
-      <c r="K9" s="4">
+        <v>750.76000000000499</v>
+      </c>
+      <c r="N9" s="4">
         <f t="shared" si="7"/>
-        <v>1065849.7600000002</v>
-      </c>
-      <c r="L9" s="4">
-        <f t="shared" si="8"/>
-        <v>-27.400000000000091</v>
-      </c>
-      <c r="M9" s="4">
-        <f t="shared" si="9"/>
-        <v>750.76000000000499</v>
-      </c>
-      <c r="N9" s="4">
-        <f t="shared" si="10"/>
         <v>4225</v>
       </c>
     </row>
@@ -3872,47 +3839,47 @@
         <v>1800</v>
       </c>
       <c r="D10" s="4">
+        <f t="shared" si="8"/>
+        <v>305</v>
+      </c>
+      <c r="E10" s="4">
         <f t="shared" si="0"/>
-        <v>305</v>
-      </c>
-      <c r="E10" s="4">
+        <v>93025</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="9"/>
+        <v>4</v>
+      </c>
+      <c r="G10" s="4">
         <f t="shared" si="1"/>
-        <v>93025</v>
-      </c>
-      <c r="F10" s="4">
+        <v>16</v>
+      </c>
+      <c r="H10" s="4">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="G10" s="4">
+        <v>1220</v>
+      </c>
+      <c r="I10" s="4">
         <f t="shared" si="3"/>
-        <v>16</v>
-      </c>
-      <c r="H10" s="4">
+        <v>1654.0000000000002</v>
+      </c>
+      <c r="J10" s="4">
+        <f t="shared" si="10"/>
+        <v>159.00000000000023</v>
+      </c>
+      <c r="K10" s="4">
         <f t="shared" si="4"/>
-        <v>1220</v>
-      </c>
-      <c r="I10" s="4">
+        <v>25281.000000000073</v>
+      </c>
+      <c r="L10" s="4">
         <f t="shared" si="5"/>
-        <v>1654.0000000000002</v>
-      </c>
-      <c r="J10" s="4">
+        <v>145.99999999999977</v>
+      </c>
+      <c r="M10" s="4">
         <f t="shared" si="6"/>
-        <v>159.00000000000023</v>
-      </c>
-      <c r="K10" s="4">
+        <v>21315.999999999935</v>
+      </c>
+      <c r="N10" s="4">
         <f t="shared" si="7"/>
-        <v>25281.000000000073</v>
-      </c>
-      <c r="L10" s="4">
-        <f t="shared" si="8"/>
-        <v>145.99999999999977</v>
-      </c>
-      <c r="M10" s="4">
-        <f t="shared" si="9"/>
-        <v>21315.999999999935</v>
-      </c>
-      <c r="N10" s="4">
-        <f t="shared" si="10"/>
         <v>1849</v>
       </c>
     </row>
@@ -3927,47 +3894,47 @@
         <v>1200</v>
       </c>
       <c r="D11" s="4">
+        <f t="shared" si="8"/>
+        <v>-295</v>
+      </c>
+      <c r="E11" s="4">
         <f t="shared" si="0"/>
-        <v>-295</v>
-      </c>
-      <c r="E11" s="4">
+        <v>87025</v>
+      </c>
+      <c r="F11" s="4">
+        <f t="shared" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="G11" s="4">
         <f t="shared" si="1"/>
-        <v>87025</v>
-      </c>
-      <c r="F11" s="4">
+        <v>81</v>
+      </c>
+      <c r="H11" s="4">
         <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
-      <c r="G11" s="4">
+        <v>-2655</v>
+      </c>
+      <c r="I11" s="4">
         <f t="shared" si="3"/>
-        <v>81</v>
-      </c>
-      <c r="H11" s="4">
+        <v>1852.5000000000002</v>
+      </c>
+      <c r="J11" s="4">
+        <f t="shared" si="10"/>
+        <v>357.50000000000023</v>
+      </c>
+      <c r="K11" s="4">
         <f t="shared" si="4"/>
-        <v>-2655</v>
-      </c>
-      <c r="I11" s="4">
+        <v>127806.25000000016</v>
+      </c>
+      <c r="L11" s="4">
         <f t="shared" si="5"/>
-        <v>1852.5000000000002</v>
-      </c>
-      <c r="J11" s="4">
+        <v>-652.50000000000023</v>
+      </c>
+      <c r="M11" s="4">
         <f t="shared" si="6"/>
-        <v>357.50000000000023</v>
-      </c>
-      <c r="K11" s="4">
+        <v>425756.25000000029</v>
+      </c>
+      <c r="N11" s="4">
         <f t="shared" si="7"/>
-        <v>127806.25000000016</v>
-      </c>
-      <c r="L11" s="4">
-        <f t="shared" si="8"/>
-        <v>-652.50000000000023</v>
-      </c>
-      <c r="M11" s="4">
-        <f t="shared" si="9"/>
-        <v>425756.25000000029</v>
-      </c>
-      <c r="N11" s="4">
-        <f t="shared" si="10"/>
         <v>2304</v>
       </c>
     </row>
@@ -4000,15 +3967,15 @@
         <v>4202250</v>
       </c>
       <c r="F14">
-        <f t="shared" ref="F14:H14" si="11">SUM(F2:F11)</f>
+        <f>SUM(F2:F11)</f>
         <v>0</v>
       </c>
       <c r="G14">
-        <f t="shared" si="11"/>
+        <f>SUM(G2:G11)</f>
         <v>2096</v>
       </c>
       <c r="H14">
-        <f t="shared" si="11"/>
+        <f>SUM(H2:H11)</f>
         <v>83200</v>
       </c>
       <c r="J14" s="5" t="s">

</xml_diff>